<commit_message>
Update website and study notes
</commit_message>
<xml_diff>
--- a/GoldfishMemory.xlsx
+++ b/GoldfishMemory.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manju\Desktop\Academia\website_portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0928EB53-6405-4FA7-A04B-27117BDCBF12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF33FB4B-1A12-40DD-AC57-D00BA3FCC66B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Neuroscience" sheetId="2" r:id="rId1"/>
-    <sheet name="Maths" sheetId="1" r:id="rId2"/>
+    <sheet name="Maths" sheetId="1" r:id="rId1"/>
+    <sheet name="Neuroscience" sheetId="2" r:id="rId2"/>
     <sheet name="Research methods" sheetId="3" r:id="rId3"/>
     <sheet name="Quiz" sheetId="4" r:id="rId4"/>
   </sheets>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="116">
   <si>
     <t>Neuroscience</t>
   </si>
@@ -271,16 +271,106 @@
     <t>Fish</t>
   </si>
   <si>
-    <t>Average</t>
-  </si>
-  <si>
-    <t>Top score</t>
-  </si>
-  <si>
     <t>Outlier</t>
   </si>
   <si>
     <t xml:space="preserve">Z normalization </t>
+  </si>
+  <si>
+    <t>Z-score normalization/standardization, is crucial data preprocessing technique in machine learning and statistics. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Converts the data into unitless numbers. The new units are standard deviations away from the mean of the distribution. Z= X−μ/ σ </t>
+  </si>
+  <si>
+    <t>Why are outliers scary?</t>
+  </si>
+  <si>
+    <t>When squared, it makes huge variation and impact on the graph</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It is not scary. </t>
+  </si>
+  <si>
+    <t>Outliers are always biased and almost never true data</t>
+  </si>
+  <si>
+    <t>The highest score</t>
+  </si>
+  <si>
+    <t>Central tendency/ the average</t>
+  </si>
+  <si>
+    <t>Why is MRI popular?</t>
+  </si>
+  <si>
+    <t>Non-invasive, non-ionizing radiation</t>
+  </si>
+  <si>
+    <t>Good spatial resolution</t>
+  </si>
+  <si>
+    <t>Superior soft tissue contrast in vivo (can show difference in tissue type)</t>
+  </si>
+  <si>
+    <t>All of the above</t>
+  </si>
+  <si>
+    <t>Fundamentals of Neuroimaging Techniques [Notes from MSc course]</t>
+  </si>
+  <si>
+    <t>Set theory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set is collection of distinct items where order does not matter and there is no repetition. {} Elements of a set need not be related at all but MUST BE WELL DEFINED. Represented as a roster listing all elements one by one {each,item,separated,by,commas} or as a a set builder form {x:followed by the condition that x follows that acts as a filter}. </t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=iTZfATpm0Yk</t>
+  </si>
+  <si>
+    <t>Types of sets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finite set, Infinite set, Equal sets, Equivalent sets (same number of element), Singleton (one element), empty/nut set (no elements), subset and superset, power sets, universal set  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basis for discrete math; also very common in coding  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow several algebraic rules. The notations are extremely annoying but commonly used. Set notation, union (∪), intersection (∩), complement ('), Cartesian product (A × B), De Morgan Laws (describe how the complement of a set interacts with the union and intersection of sets.). Helpful to google 'set theory notation cheat sheet. </t>
+  </si>
+  <si>
+    <t>Intervals</t>
+  </si>
+  <si>
+    <t>A connected subset of numbers containing all numbers that lie between two designated endpoints a and b (where a &lt; b).</t>
+  </si>
+  <si>
+    <t>Open Interval (a, b), Closed Interval [a, b], Half-Open / Half-Closed Interval: Includes only one endpoint [a, b) or (a, b], Infinite Interval [a, ∞) or (-∞, b].</t>
+  </si>
+  <si>
+    <t>https://youtu.be/zpln5ExhkyI?si=FCetaqTdXNPH_zlQ   ; https://www.geeksforgeeks.org/maths/absolute-value/</t>
+  </si>
+  <si>
+    <t>Absolute value</t>
+  </si>
+  <si>
+    <t>bsolute value of a number represents its distance from zero on the number line, regardless of direction. It is always non-negative</t>
+  </si>
+  <si>
+    <t>denote by |x|</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>https://youtu.be/52tpYl2tTqk?si=fuH3EUDmCFAeFrVI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explains how one set relates to another. Input set (domain) and output set (range). Sort of a machine that takes an input x and gives you exactly one output f(x). One input cannot give 2 outputs.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Has specific arithmetic rules that it follows. Especially with the second set. </t>
   </si>
 </sst>
 </file>
@@ -462,7 +552,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -531,12 +621,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -680,6 +807,46 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -697,34 +864,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -746,6 +885,10 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -962,121 +1105,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="20" style="28" customWidth="1"/>
-    <col min="2" max="2" width="46" style="28" customWidth="1"/>
-    <col min="3" max="3" width="44.6328125" style="28" customWidth="1"/>
-    <col min="4" max="4" width="47.7265625" style="28" customWidth="1"/>
-    <col min="5" max="5" width="21.26953125" style="28" customWidth="1"/>
-    <col min="6" max="16384" width="12.6328125" style="26"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" s="23" customFormat="1" ht="15.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-    </row>
-    <row r="2" spans="1:5" s="23" customFormat="1" ht="13" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="24"/>
-    </row>
-    <row r="3" spans="1:5" s="25" customFormat="1" ht="13" x14ac:dyDescent="0.25">
-      <c r="A3" s="41" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="43"/>
-    </row>
-    <row r="4" spans="1:5" ht="50" x14ac:dyDescent="0.25">
-      <c r="A4" s="27" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="28" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="B5" s="27" t="s">
-        <v>55</v>
-      </c>
-      <c r="C5" s="27" t="s">
-        <v>56</v>
-      </c>
-      <c r="D5" s="28" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="46" customFormat="1" ht="13" x14ac:dyDescent="0.25">
-      <c r="A6" s="44" t="s">
-        <v>43</v>
-      </c>
-      <c r="B6" s="45"/>
-      <c r="C6" s="45"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-    </row>
-    <row r="7" spans="1:5" ht="50" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="B7" s="27" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" s="27" t="s">
-        <v>52</v>
-      </c>
-      <c r="D7" s="28" t="s">
-        <v>51</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A6:XFD6"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" style="10" customWidth="1"/>
@@ -1115,12 +1149,12 @@
       <c r="F2" s="17"/>
     </row>
     <row r="3" spans="1:6" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.25">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
       <c r="E3" s="13"/>
       <c r="F3" s="18"/>
     </row>
@@ -1157,211 +1191,413 @@
       <c r="F5" s="19"/>
     </row>
     <row r="6" spans="1:6" ht="75" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="14"/>
+      <c r="E6" s="43"/>
       <c r="F6" s="19"/>
     </row>
-    <row r="7" spans="1:6" s="50" customFormat="1" ht="13" x14ac:dyDescent="0.25">
-      <c r="A7" s="48" t="s">
+    <row r="7" spans="1:6" ht="87.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="41" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" s="41" t="s">
+        <v>99</v>
+      </c>
+      <c r="C7" s="41" t="s">
+        <v>103</v>
+      </c>
+      <c r="D7" s="42" t="s">
+        <v>100</v>
+      </c>
+      <c r="E7" s="43"/>
+      <c r="F7" s="19"/>
+    </row>
+    <row r="8" spans="1:6" ht="87.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="41" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" s="41" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" s="42" t="s">
+        <v>100</v>
+      </c>
+      <c r="E8" s="43"/>
+      <c r="F8" s="19"/>
+    </row>
+    <row r="9" spans="1:6" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="41" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" s="41" t="s">
+        <v>106</v>
+      </c>
+      <c r="C9" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="D9" s="42"/>
+      <c r="E9" s="43"/>
+      <c r="F9" s="19"/>
+    </row>
+    <row r="10" spans="1:6" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="41" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" s="41" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" s="41" t="s">
+        <v>111</v>
+      </c>
+      <c r="D10" s="42" t="s">
+        <v>108</v>
+      </c>
+      <c r="E10" s="43"/>
+      <c r="F10" s="19"/>
+    </row>
+    <row r="11" spans="1:6" ht="50" x14ac:dyDescent="0.25">
+      <c r="A11" s="41" t="s">
+        <v>112</v>
+      </c>
+      <c r="B11" s="41" t="s">
+        <v>114</v>
+      </c>
+      <c r="C11" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="D11" s="64" t="s">
+        <v>113</v>
+      </c>
+      <c r="E11" s="43"/>
+      <c r="F11" s="19"/>
+    </row>
+    <row r="12" spans="1:6" s="47" customFormat="1" ht="13" x14ac:dyDescent="0.25">
+      <c r="A12" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-    </row>
-    <row r="8" spans="1:6" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="B12" s="46"/>
+      <c r="C12" s="46"/>
+      <c r="D12" s="46"/>
+      <c r="E12" s="46"/>
+      <c r="F12" s="46"/>
+    </row>
+    <row r="13" spans="1:6" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B13" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C13" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="30" t="s">
+      <c r="D13" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="14"/>
-      <c r="F8" s="19"/>
-    </row>
-    <row r="9" spans="1:6" ht="50" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="E13" s="14"/>
+      <c r="F13" s="19"/>
+    </row>
+    <row r="14" spans="1:6" ht="50" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B14" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C14" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="31" t="s">
+      <c r="D14" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="14"/>
-      <c r="F9" s="19"/>
-    </row>
-    <row r="10" spans="1:6" ht="25" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" s="14"/>
-      <c r="F10" s="19"/>
-    </row>
-    <row r="11" spans="1:6" ht="25" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E11" s="14"/>
-      <c r="F11" s="19"/>
-    </row>
-    <row r="12" spans="1:6" ht="25" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E12" s="14"/>
-      <c r="F12" s="19"/>
-    </row>
-    <row r="13" spans="1:6" s="53" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="51" t="s">
-        <v>62</v>
-      </c>
-      <c r="B13" s="52"/>
-      <c r="C13" s="52"/>
-      <c r="D13" s="52"/>
-      <c r="E13" s="52"/>
-      <c r="F13" s="52"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="D14" s="9"/>
       <c r="E14" s="14"/>
       <c r="F14" s="19"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
+    <row r="15" spans="1:6" ht="25" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>34</v>
+      </c>
       <c r="E15" s="14"/>
       <c r="F15" s="19"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
+    <row r="16" spans="1:6" ht="25" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>51</v>
+      </c>
       <c r="E16" s="14"/>
       <c r="F16" s="19"/>
     </row>
-    <row r="17" spans="1:6" ht="87.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
-        <v>66</v>
+    <row r="17" spans="1:6" ht="25" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>48</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D17" s="9"/>
+        <v>50</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>51</v>
+      </c>
       <c r="E17" s="14"/>
       <c r="F17" s="19"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="19"/>
+    <row r="18" spans="1:6" s="50" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="48" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" s="49"/>
+      <c r="C18" s="49"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="49"/>
+      <c r="F18" s="49"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
+      <c r="A19" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>58</v>
+      </c>
       <c r="D19" s="9"/>
       <c r="E19" s="14"/>
       <c r="F19" s="19"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
+      <c r="A20" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>63</v>
+      </c>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
       <c r="E20" s="14"/>
       <c r="F20" s="19"/>
     </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="19"/>
+    </row>
+    <row r="22" spans="1:6" ht="87.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D22" s="9"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="19"/>
+    </row>
+    <row r="23" spans="1:6" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A23" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D23" s="9"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="19"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="9"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="19"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="9"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="19"/>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A7:XFD7"/>
-    <mergeCell ref="A13:XFD13"/>
+    <mergeCell ref="A12:XFD12"/>
+    <mergeCell ref="A18:XFD18"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D5" r:id="rId1" xr:uid="{92139182-3192-4FD1-B073-C33397C80744}"/>
-    <hyperlink ref="D9" r:id="rId2" xr:uid="{D1A1E46E-289A-40F9-8E46-65C6381295A3}"/>
+    <hyperlink ref="D14" r:id="rId2" xr:uid="{D1A1E46E-289A-40F9-8E46-65C6381295A3}"/>
+    <hyperlink ref="D11" r:id="rId3" xr:uid="{32425B40-8980-4DFC-B5ED-4064E201972D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="44" fitToHeight="0" orientation="portrait" r:id="rId3"/>
+  <pageSetup scale="44" fitToHeight="0" orientation="portrait" r:id="rId4"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20" style="28" customWidth="1"/>
+    <col min="2" max="2" width="46" style="28" customWidth="1"/>
+    <col min="3" max="3" width="44.6328125" style="28" customWidth="1"/>
+    <col min="4" max="4" width="47.7265625" style="28" customWidth="1"/>
+    <col min="5" max="5" width="21.26953125" style="28" customWidth="1"/>
+    <col min="6" max="16384" width="12.6328125" style="26"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="23" customFormat="1" ht="15.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+    </row>
+    <row r="2" spans="1:5" s="23" customFormat="1" ht="13" x14ac:dyDescent="0.25">
+      <c r="A2" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="24"/>
+    </row>
+    <row r="3" spans="1:5" s="25" customFormat="1" ht="13" x14ac:dyDescent="0.25">
+      <c r="A3" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="52"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="52"/>
+      <c r="E3" s="53"/>
+    </row>
+    <row r="4" spans="1:5" ht="50" x14ac:dyDescent="0.25">
+      <c r="A4" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="28" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="28" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="56" customFormat="1" ht="13" x14ac:dyDescent="0.25">
+      <c r="A6" s="54" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+    </row>
+    <row r="7" spans="1:5" ht="50" x14ac:dyDescent="0.25">
+      <c r="A7" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="28" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" s="56" customFormat="1" ht="13" x14ac:dyDescent="0.25">
+      <c r="A8" s="54" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="55"/>
+      <c r="C8" s="55"/>
+      <c r="D8" s="55"/>
+      <c r="E8" s="55"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A6:XFD6"/>
+    <mergeCell ref="A8:XFD8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1383,14 +1619,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="32" customFormat="1" ht="13.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
     </row>
     <row r="2" spans="1:6" s="32" customFormat="1" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
@@ -1409,14 +1645,14 @@
       <c r="F2" s="33"/>
     </row>
     <row r="3" spans="1:6" s="34" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
     </row>
     <row r="4" spans="1:6" ht="25" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
@@ -1433,15 +1669,15 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:6" s="60" customFormat="1" ht="13" x14ac:dyDescent="0.3">
-      <c r="A7" s="58" t="s">
+    <row r="7" spans="1:6" s="63" customFormat="1" ht="13" x14ac:dyDescent="0.3">
+      <c r="A7" s="61" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="59"/>
-      <c r="C7" s="59"/>
-      <c r="D7" s="59"/>
-      <c r="E7" s="59"/>
-      <c r="F7" s="59"/>
+      <c r="B7" s="62"/>
+      <c r="C7" s="62"/>
+      <c r="D7" s="62"/>
+      <c r="E7" s="62"/>
+      <c r="F7" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1455,7 +1691,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C239A2E7-9F6A-46E7-89C3-299758E3487A}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.26953125" style="40" customWidth="1"/>
@@ -1513,17 +1749,51 @@
       <c r="B3" s="40" t="s">
         <v>81</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="39" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="E3" s="40" t="s">
         <v>82</v>
-      </c>
-      <c r="D3" s="40" t="s">
-        <v>83</v>
-      </c>
-      <c r="E3" s="40" t="s">
-        <v>84</v>
       </c>
       <c r="F3" s="40" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="25" x14ac:dyDescent="0.25">
+      <c r="A4" s="39" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="39" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" s="39" t="s">
+        <v>88</v>
+      </c>
+      <c r="D4" s="39" t="s">
+        <v>89</v>
+      </c>
+      <c r="F4" s="39" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="39" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" s="39" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" s="39" t="s">
+        <v>94</v>
+      </c>
+      <c r="D5" s="39" t="s">
+        <v>95</v>
+      </c>
+      <c r="E5" s="39" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>